<commit_message>
Fixed a bug in the weighing of topk vs remainder entropies. Introduced the dashboard of CRN topologies. Plotting folder added.
</commit_message>
<xml_diff>
--- a/apps_Maurice_MAK_REINFORCE/RPA_6species_6rxns/RPA_6species_6rxns_MAK_REINFORCE.xlsx
+++ b/apps_Maurice_MAK_REINFORCE/RPA_6species_6rxns/RPA_6species_6rxns_MAK_REINFORCE.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="38">
   <si>
     <t>Timestamp</t>
   </si>
@@ -22,12 +22,18 @@
     <t>2025-11-17 13:11:10</t>
   </si>
   <si>
+    <t>2025-11-23 01:01:57</t>
+  </si>
+  <si>
     <t>URL</t>
   </si>
   <si>
     <t>https://www.comet.com/maurice-filo/rpa-6species-6rxns-mak-reinforce/b6f58fef17a94499a09db4f965b765c4</t>
   </si>
   <si>
+    <t>https://www.comet.com/maurice-filo/rpa-6species-6rxns-mak-reinforce/3777fccb482e4a359b591eb2f0f9c4fd</t>
+  </si>
+  <si>
     <t>Maximum Number of Added Reactions</t>
   </si>
   <si>
@@ -101,6 +107,9 @@
   </si>
   <si>
     <t>{'structure': 1.0, 'continuous': 0.1, 'discrete': 0.0, 'input_influence': 0.0}</t>
+  </si>
+  <si>
+    <t>{'structure': 1.0, 'continuous': 0.5, 'discrete': 0.0, 'input_influence': 0.0}</t>
   </si>
   <si>
     <t>Epochs Completed</t>
@@ -136,13 +145,13 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -174,7 +183,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -182,20 +191,29 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -502,228 +520,302 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="28.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="28.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="9" width="28.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="10" width="28.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="11" width="29.290714285714284" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="4">
+        <v>8</v>
+      </c>
+      <c r="C3" s="5">
+        <v>8</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="4">
+        <v>6</v>
+      </c>
+      <c r="C4" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
-      <c r="A3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="3">
-        <v>8</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="1" t="s">
+      <c r="C5" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="4">
+        <v>1280</v>
+      </c>
+      <c r="C6" s="5">
+        <v>1280</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="7">
+        <v>0.0001</v>
+      </c>
+      <c r="C8" s="8">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="A9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="4">
+        <v>300</v>
+      </c>
+      <c r="C9" s="5">
+        <v>300</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+      <c r="A10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="4">
         <v>5</v>
       </c>
-      <c r="B4" s="3">
-        <v>6</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="3">
-        <v>3</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
-      <c r="A6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="3">
-        <v>1280</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
-      <c r="A7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
-      <c r="A8" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="5">
-        <v>0.0001</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
-      <c r="A9" s="1" t="s">
+      <c r="C10" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+      <c r="A11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="4">
+        <v>1024</v>
+      </c>
+      <c r="C11" s="5">
+        <v>1024</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+      <c r="A12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="4">
+        <v>10240</v>
+      </c>
+      <c r="C12" s="5">
+        <v>10240</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+      <c r="A13" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="4">
+        <v>128</v>
+      </c>
+      <c r="C13" s="5">
+        <v>128</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+      <c r="A14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+      <c r="A15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+      <c r="A16" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="4">
         <v>10</v>
       </c>
-      <c r="B9" s="3">
-        <v>300</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
-      <c r="A10" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" s="3">
-        <v>5</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
-      <c r="A11" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="3">
-        <v>1024</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
-      <c r="A12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="3">
-        <v>10240</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
-      <c r="A13" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" s="3">
-        <v>128</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
-      <c r="A14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
-      <c r="A15" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
-      <c r="A16" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16" s="3">
+      <c r="C16" s="5">
         <v>10</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="4">
         <v>20</v>
       </c>
-      <c r="B17" s="3">
+      <c r="C17" s="5">
         <v>20</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="3">
+        <v>23</v>
+      </c>
+      <c r="B18" s="4">
+        <v>200</v>
+      </c>
+      <c r="C18" s="5">
         <v>200</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
       <c r="A19" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19" s="3">
+        <v>24</v>
+      </c>
+      <c r="B19" s="4">
+        <v>1000</v>
+      </c>
+      <c r="C19" s="5">
         <v>1000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25">
       <c r="A20" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B20" s="3">
+        <v>25</v>
+      </c>
+      <c r="B20" s="4">
+        <v>1</v>
+      </c>
+      <c r="C20" s="5">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="17.25">
       <c r="A21" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B21" s="3">
+        <v>26</v>
+      </c>
+      <c r="B21" s="4">
+        <v>27</v>
+      </c>
+      <c r="C21" s="5">
         <v>27</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="17.25">
       <c r="A22" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="17.25">
       <c r="A23" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>31</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="17.25">
       <c r="A24" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>30</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="17.25">
       <c r="A25" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>30</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="17.25">
       <c r="A26" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>30</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="17.25">
       <c r="A27" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>34</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C27" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>